<commit_message>
Fix a bug in matching (when we have a single term, we accidentally consider it as a list of term) + change prompt to prevent hallucinate from examples + output as json for better integration with llm + fix certain info like cohorts to not have examples in llm prompt to prevent hallucination
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_37002253_table5_v1.xlsx
+++ b/harmonized_tables_advp/from_37002253_table5_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT18"/>
+  <dimension ref="A1:AU18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,85 +576,90 @@
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
+          <t>P-value note</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
           <t>BP(Position)</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>RA 1(Reported Allele 1)</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>RA 2(Reported Allele 2)</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Note on alleles and AF</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>ReportedAF(MAF)</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>AFincases</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>AFincontrols</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Effect Size Type (OR or Beta)</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>EffectSize(altvsref)</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>95%ConfidenceInterval</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Confirmed affected genes, causal variants, evidence</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Genome build (hg18/hg37/hg38)</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Pubmed PMID</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>PMCID</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Table Ref in paper</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Table links</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>LocusName</t>
         </is>
@@ -685,7 +690,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -696,7 +701,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
@@ -704,19 +713,19 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -736,49 +745,50 @@
       <c r="AC2" t="n">
         <v>0.004</v>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr">
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL2" t="n">
-        <v>0.044</v>
-      </c>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AM2" t="n">
+        <v>-0.044</v>
+      </c>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr">
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Bacteroi</t>
         </is>
@@ -809,7 +819,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -820,7 +830,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
@@ -828,19 +842,19 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -860,49 +874,50 @@
       <c r="AC3" t="n">
         <v>0.025</v>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr">
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL3" t="n">
-        <v>0.044</v>
-      </c>
-      <c r="AM3" t="inlineStr"/>
+      <c r="AM3" t="n">
+        <v>-0.044</v>
+      </c>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr">
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ3" t="inlineStr">
+      <c r="AR3" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS3" t="inlineStr">
+      <c r="AT3" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t>Butyricimo</t>
         </is>
@@ -933,7 +948,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -944,7 +959,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -952,19 +971,19 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -984,49 +1003,50 @@
       <c r="AC4" t="n">
         <v>0.0334</v>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr">
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL4" t="n">
+      <c r="AM4" t="n">
         <v>0.03</v>
       </c>
-      <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr">
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr">
+      <c r="AR4" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS4" t="inlineStr">
+      <c r="AT4" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr">
+      <c r="AU4" t="inlineStr">
         <is>
           <t>Do</t>
         </is>
@@ -1057,7 +1077,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1068,7 +1088,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
@@ -1076,19 +1100,19 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -1108,49 +1132,50 @@
       <c r="AC5" t="n">
         <v>0.034</v>
       </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr">
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL5" t="n">
+      <c r="AM5" t="n">
         <v>0.033</v>
       </c>
-      <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr">
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr">
+      <c r="AR5" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR5" t="inlineStr">
+      <c r="AS5" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS5" t="inlineStr">
+      <c r="AT5" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr">
+      <c r="AU5" t="inlineStr">
         <is>
           <t>Eubacter coprostanolige</t>
         </is>
@@ -1181,7 +1206,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1192,7 +1217,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
@@ -1200,19 +1229,19 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -1232,49 +1261,50 @@
       <c r="AC6" t="n">
         <v>0.0287</v>
       </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr">
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL6" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="AM6" t="inlineStr"/>
+      <c r="AM6" t="n">
+        <v>-0.035</v>
+      </c>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr">
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ6" t="inlineStr">
+      <c r="AR6" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AS6" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS6" t="inlineStr">
+      <c r="AT6" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT6" t="inlineStr">
+      <c r="AU6" t="inlineStr">
         <is>
           <t>Faecalibacter</t>
         </is>
@@ -1305,7 +1335,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1316,7 +1346,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
@@ -1324,19 +1358,19 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1356,49 +1390,50 @@
       <c r="AC7" t="n">
         <v>0.0462</v>
       </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr">
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL7" t="n">
+      <c r="AM7" t="n">
         <v>0.064</v>
       </c>
-      <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr">
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr">
+      <c r="AR7" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr">
+      <c r="AS7" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
+      <c r="AT7" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT7" t="inlineStr">
+      <c r="AU7" t="inlineStr">
         <is>
           <t>Olsene</t>
         </is>
@@ -1429,7 +1464,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1440,7 +1475,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
@@ -1448,19 +1487,19 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1480,49 +1519,50 @@
       <c r="AC8" t="n">
         <v>0.0267</v>
       </c>
-      <c r="AD8" t="inlineStr">
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr">
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL8" t="n">
+      <c r="AM8" t="n">
         <v>0.04</v>
       </c>
-      <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr">
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AR8" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr">
+      <c r="AS8" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS8" t="inlineStr">
+      <c r="AT8" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT8" t="inlineStr">
+      <c r="AU8" t="inlineStr">
         <is>
           <t>Parasuttere</t>
         </is>
@@ -1553,7 +1593,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1564,7 +1604,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
@@ -1572,19 +1616,19 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1604,49 +1648,50 @@
       <c r="AC9" t="n">
         <v>0.0273</v>
       </c>
-      <c r="AD9" t="inlineStr">
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr">
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL9" t="n">
+      <c r="AM9" t="n">
         <v>0.05</v>
       </c>
-      <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
-      <c r="AP9" t="inlineStr">
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ9" t="inlineStr">
+      <c r="AR9" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr">
+      <c r="AS9" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS9" t="inlineStr">
+      <c r="AT9" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT9" t="inlineStr">
+      <c r="AU9" t="inlineStr">
         <is>
           <t>Senegalimassi</t>
         </is>
@@ -1677,7 +1722,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1688,7 +1733,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
@@ -1696,19 +1745,19 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1728,49 +1777,50 @@
       <c r="AC10" t="n">
         <v>0.0421</v>
       </c>
-      <c r="AD10" t="inlineStr">
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr">
         <is>
           <t>rs429358 (19:45411941:C)</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr">
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL10" t="n">
+      <c r="AM10" t="n">
         <v>0.044</v>
       </c>
-      <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
-      <c r="AP10" t="inlineStr">
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ10" t="inlineStr">
+      <c r="AR10" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR10" t="inlineStr">
+      <c r="AS10" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS10" t="inlineStr">
+      <c r="AT10" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT10" t="inlineStr">
+      <c r="AU10" t="inlineStr">
         <is>
           <t>Veillone</t>
         </is>
@@ -1801,7 +1851,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1812,7 +1862,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
@@ -1820,19 +1874,19 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1852,49 +1906,50 @@
       <c r="AC11" t="n">
         <v>0.0136</v>
       </c>
-      <c r="AD11" t="inlineStr">
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr">
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL11" t="n">
+      <c r="AM11" t="n">
         <v>0.048</v>
       </c>
-      <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
-      <c r="AP11" t="inlineStr">
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ11" t="inlineStr">
+      <c r="AR11" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR11" t="inlineStr">
+      <c r="AS11" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS11" t="inlineStr">
+      <c r="AT11" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT11" t="inlineStr">
+      <c r="AU11" t="inlineStr">
         <is>
           <t>Butyricicoc</t>
         </is>
@@ -1925,7 +1980,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1936,7 +1991,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
@@ -1944,19 +2003,19 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1976,49 +2035,50 @@
       <c r="AC12" t="n">
         <v>0.0268</v>
       </c>
-      <c r="AD12" t="inlineStr">
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="inlineStr"/>
       <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr">
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL12" t="n">
+      <c r="AM12" t="n">
         <v>0.052</v>
       </c>
-      <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr">
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ12" t="inlineStr">
+      <c r="AR12" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR12" t="inlineStr">
+      <c r="AS12" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS12" t="inlineStr">
+      <c r="AT12" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT12" t="inlineStr">
+      <c r="AU12" t="inlineStr">
         <is>
           <t>Collinse</t>
         </is>
@@ -2049,7 +2109,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2060,7 +2120,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
@@ -2068,19 +2132,19 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -2100,49 +2164,50 @@
       <c r="AC13" t="n">
         <v>0.0191</v>
       </c>
-      <c r="AD13" t="inlineStr">
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr">
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL13" t="n">
+      <c r="AM13" t="n">
         <v>0.05</v>
       </c>
-      <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr">
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ13" t="inlineStr">
+      <c r="AR13" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR13" t="inlineStr">
+      <c r="AS13" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS13" t="inlineStr">
+      <c r="AT13" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT13" t="inlineStr">
+      <c r="AU13" t="inlineStr">
         <is>
           <t>Coprococcus3</t>
         </is>
@@ -2173,7 +2238,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2184,7 +2249,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -2192,19 +2261,19 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -2224,49 +2293,50 @@
       <c r="AC14" t="n">
         <v>0.0142</v>
       </c>
-      <c r="AD14" t="inlineStr">
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
       <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr">
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL14" t="n">
+      <c r="AM14" t="n">
         <v>0.053</v>
       </c>
-      <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
-      <c r="AP14" t="inlineStr">
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ14" t="inlineStr">
+      <c r="AR14" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR14" t="inlineStr">
+      <c r="AS14" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS14" t="inlineStr">
+      <c r="AT14" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT14" t="inlineStr">
+      <c r="AU14" t="inlineStr">
         <is>
           <t>Eubacter hal</t>
         </is>
@@ -2297,7 +2367,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2308,7 +2378,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
@@ -2316,19 +2390,19 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -2348,49 +2422,50 @@
       <c r="AC15" t="n">
         <v>0.0113</v>
       </c>
-      <c r="AD15" t="inlineStr">
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr">
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL15" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="AM15" t="inlineStr"/>
+      <c r="AM15" t="n">
+        <v>-0.07099999999999999</v>
+      </c>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
-      <c r="AP15" t="inlineStr">
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ15" t="inlineStr">
+      <c r="AR15" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR15" t="inlineStr">
+      <c r="AS15" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS15" t="inlineStr">
+      <c r="AT15" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT15" t="inlineStr">
+      <c r="AU15" t="inlineStr">
         <is>
           <t>Lachnospirac UCG001</t>
         </is>
@@ -2421,7 +2496,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2432,7 +2507,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
@@ -2440,19 +2519,19 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -2472,49 +2551,50 @@
       <c r="AC16" t="n">
         <v>0.019</v>
       </c>
-      <c r="AD16" t="inlineStr">
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="inlineStr"/>
       <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr">
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL16" t="n">
-        <v>0.103</v>
-      </c>
-      <c r="AM16" t="inlineStr"/>
+      <c r="AM16" t="n">
+        <v>-0.103</v>
+      </c>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr">
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ16" t="inlineStr">
+      <c r="AR16" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR16" t="inlineStr">
+      <c r="AS16" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS16" t="inlineStr">
+      <c r="AT16" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT16" t="inlineStr">
+      <c r="AU16" t="inlineStr">
         <is>
           <t>Olsene</t>
         </is>
@@ -2545,7 +2625,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2556,7 +2636,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
@@ -2564,19 +2648,19 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -2596,49 +2680,50 @@
       <c r="AC17" t="n">
         <v>0.0037</v>
       </c>
-      <c r="AD17" t="inlineStr">
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr"/>
       <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr">
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL17" t="n">
+      <c r="AM17" t="n">
         <v>0.08</v>
       </c>
-      <c r="AM17" t="inlineStr"/>
       <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr"/>
-      <c r="AP17" t="inlineStr">
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ17" t="inlineStr">
+      <c r="AR17" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR17" t="inlineStr">
+      <c r="AS17" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS17" t="inlineStr">
+      <c r="AT17" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT17" t="inlineStr">
+      <c r="AU17" t="inlineStr">
         <is>
           <t>Ruminococcac UCG004</t>
         </is>
@@ -2669,7 +2754,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>discovery + meta-analysis + Meta-analysis + replication</t>
+          <t>replication + discovery + meta-analysis</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -2680,7 +2765,11 @@
           <t>SNP-based</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>igap + adgc + niaload + adni + charge + genada + mibiogen + eadi + uk biobank</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
@@ -2688,19 +2777,19 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UK10K + TOPMed + 1000G + HRC + minimac4</t>
+          <t>michigan imputation server minimac4 + 1000 genome phase 3v5</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>EUR + middle-east + EAS + AA + hispanic + European ancestry + african american</t>
+          <t>eur + european ancestry + hispanic + eas + aa</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Genada + ADC12 + NIALOAD + UA + AD</t>
+          <t>alzheimers disease + ad</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -2720,49 +2809,50 @@
       <c r="AC18" t="n">
         <v>0.0098</v>
       </c>
-      <c r="AD18" t="inlineStr">
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr">
         <is>
           <t>rs7412 (19:45412079:T)</t>
         </is>
       </c>
-      <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr"/>
       <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr">
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="AL18" t="n">
+      <c r="AM18" t="n">
         <v>0.082</v>
       </c>
-      <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="inlineStr">
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr">
         <is>
           <t>37002253</t>
         </is>
       </c>
-      <c r="AQ18" t="inlineStr">
+      <c r="AR18" t="inlineStr">
         <is>
           <t>PMC10066300</t>
         </is>
       </c>
-      <c r="AR18" t="inlineStr">
+      <c r="AS18" t="inlineStr">
         <is>
           <t>Table 5</t>
         </is>
       </c>
-      <c r="AS18" t="inlineStr">
+      <c r="AT18" t="inlineStr">
         <is>
           <t>37002253_table5.xlsx</t>
         </is>
       </c>
-      <c r="AT18" t="inlineStr">
+      <c r="AU18" t="inlineStr">
         <is>
           <t>Senegalimassi</t>
         </is>

</xml_diff>